<commit_message>
Preserve confirmed posts when Messages notifications fail
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -393,22 +393,31 @@
         <v>long</v>
       </c>
       <c r="E3" t="str">
-        <v>pending</v>
+        <v>posted</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-07-28T00:23:09.403Z</v>
+      </c>
+      <c r="G3" t="str">
+        <v>2026-07-28T00:35:42.400Z</v>
+      </c>
+      <c r="H3" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0002-website-redesign-checklist-15-steps-before-you-hire.md</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>approved</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>YES 2 / NO 2</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>openai/gpt-oss-20b</v>
       </c>
       <c r="L3" t="str">
-        <v/>
+        <v>28351</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28351</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
@@ -425,7 +434,22 @@
         <v>medium</v>
       </c>
       <c r="E4" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-07-28T00:26:46.795Z</v>
+      </c>
+      <c r="H4" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0003-web-design-vs-web-development.md</v>
+      </c>
+      <c r="I4" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J4" t="str">
+        <v>YES 3 / NO 3</v>
+      </c>
+      <c r="K4" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
@@ -3906,15 +3930,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="11.83203125" customWidth="1"/>
-    <col min="4" max="4" width="48.83203125" customWidth="1"/>
-    <col min="5" max="5" width="64.83203125" customWidth="1"/>
-    <col min="6" max="6" width="56.83203125" customWidth="1"/>
-    <col min="7" max="7" width="44.83203125" customWidth="1"/>
-    <col min="8" max="8" width="36.83203125" customWidth="1"/>
-    <col min="9" max="9" width="48.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="30.83203125"/>
+    <col min="3" max="3" customWidth="1" width="11.83203125"/>
+    <col min="4" max="4" customWidth="1" width="48.83203125"/>
+    <col min="5" max="5" customWidth="1" width="64.83203125"/>
+    <col min="6" max="6" customWidth="1" width="56.83203125"/>
+    <col min="7" max="7" customWidth="1" width="44.83203125"/>
+    <col min="8" max="8" customWidth="1" width="36.83203125"/>
+    <col min="9" max="9" customWidth="1" width="48.83203125"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">

</xml_diff>

<commit_message>
Deliver macOS review drafts as text attachments
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -466,7 +466,22 @@
         <v>long</v>
       </c>
       <c r="E5" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-07-28T01:56:25.929Z</v>
+      </c>
+      <c r="H5" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0004-custom-website-cost-practical-budgeting-guide.md</v>
+      </c>
+      <c r="I5" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J5" t="str">
+        <v>YES 4 / NO 4</v>
+      </c>
+      <c r="K5" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">

</xml_diff>

<commit_message>
Record current blog workflow state
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -466,22 +466,31 @@
         <v>long</v>
       </c>
       <c r="E5" t="str">
-        <v>awaiting_review</v>
+        <v>posted</v>
       </c>
       <c r="F5" t="str">
         <v>2026-07-28T01:56:25.929Z</v>
       </c>
+      <c r="G5" t="str">
+        <v>2026-07-28T02:33:55.284Z</v>
+      </c>
       <c r="H5" t="str">
         <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0004-custom-website-cost-practical-budgeting-guide.md</v>
       </c>
       <c r="I5" t="str">
-        <v>pending</v>
+        <v>approved</v>
       </c>
       <c r="J5" t="str">
         <v>YES 4 / NO 4</v>
       </c>
       <c r="K5" t="str">
         <v>openai/gpt-oss-20b</v>
+      </c>
+      <c r="L5" t="str">
+        <v>28352</v>
+      </c>
+      <c r="M5" t="str">
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28352</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -498,7 +507,22 @@
         <v>medium</v>
       </c>
       <c r="E6" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2026-07-28T02:35:29.675Z</v>
+      </c>
+      <c r="H6" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0005-website-planning-checklist.md</v>
+      </c>
+      <c r="I6" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J6" t="str">
+        <v>YES 5 / NO 5</v>
+      </c>
+      <c r="K6" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -515,7 +539,22 @@
         <v>long</v>
       </c>
       <c r="E7" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F7" t="str">
+        <v>2026-07-28T02:39:48.534Z</v>
+      </c>
+      <c r="H7" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0006-conversion-focused-website-design.md</v>
+      </c>
+      <c r="I7" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J7" t="str">
+        <v>YES 6 / NO 6</v>
+      </c>
+      <c r="K7" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
@@ -532,7 +571,22 @@
         <v>medium</v>
       </c>
       <c r="E8" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F8" t="str">
+        <v>2026-07-28T02:42:43.615Z</v>
+      </c>
+      <c r="H8" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0007-b2b-website-design-best-practices.md</v>
+      </c>
+      <c r="I8" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J8" t="str">
+        <v>YES 7 / NO 7</v>
+      </c>
+      <c r="K8" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -549,7 +603,22 @@
         <v>short</v>
       </c>
       <c r="E9" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F9" t="str">
+        <v>2026-07-28T02:44:47.751Z</v>
+      </c>
+      <c r="H9" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0008-website-navigation-best-practices-build-menus-that-help-user.md</v>
+      </c>
+      <c r="I9" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J9" t="str">
+        <v>YES 8 / NO 8</v>
+      </c>
+      <c r="K9" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
@@ -566,7 +635,22 @@
         <v>medium</v>
       </c>
       <c r="E10" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F10" t="str">
+        <v>2026-07-28T02:47:44.815Z</v>
+      </c>
+      <c r="H10" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0009-website-accessibility-checklist-business-websites.md</v>
+      </c>
+      <c r="I10" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J10" t="str">
+        <v>YES 9 / NO 9</v>
+      </c>
+      <c r="K10" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
@@ -583,7 +667,22 @@
         <v>long</v>
       </c>
       <c r="E11" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F11" t="str">
+        <v>2026-07-28T02:51:01.511Z</v>
+      </c>
+      <c r="H11" t="str">
+        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0010-custom-wordpress-development-vs-page-builders.md</v>
+      </c>
+      <c r="I11" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J11" t="str">
+        <v>YES 10 / NO 10</v>
+      </c>
+      <c r="K11" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -600,6 +699,9 @@
         <v>long</v>
       </c>
       <c r="E12" t="str">
+        <v>generating</v>
+      </c>
+      <c r="I12" t="str">
         <v>pending</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update WordPress blog content tracker
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -38,11 +38,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="200" formatCode="0"/>
-    <numFmt numFmtId="201" formatCode="yyyy-mm-dd hh:mm"/>
-    <numFmt numFmtId="202" formatCode="#,##0"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -75,9 +73,9 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -275,6 +273,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -719,7 +719,22 @@
         <v>medium</v>
       </c>
       <c r="E13" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F13" t="str">
+        <v>2026-07-28T15:37:56.579Z</v>
+      </c>
+      <c r="H13" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0012-choose-wordpress-development-agency.md</v>
+      </c>
+      <c r="I13" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J13" t="str">
+        <v>YES 12 / NO 12</v>
+      </c>
+      <c r="K13" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
@@ -736,7 +751,22 @@
         <v>medium</v>
       </c>
       <c r="E14" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F14" t="str">
+        <v>2026-07-28T15:40:46.445Z</v>
+      </c>
+      <c r="H14" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0013-wordpress-security-best-practices-business-websites.md</v>
+      </c>
+      <c r="I14" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J14" t="str">
+        <v>YES 13 / NO 13</v>
+      </c>
+      <c r="K14" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
@@ -753,7 +783,22 @@
         <v>long</v>
       </c>
       <c r="E15" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F15" t="str">
+        <v>2026-07-28T15:43:28.448Z</v>
+      </c>
+      <c r="H15" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0014-wordpress-website-faster-core-web-vitals-guide.md</v>
+      </c>
+      <c r="I15" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J15" t="str">
+        <v>YES 14 / NO 14</v>
+      </c>
+      <c r="K15" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
@@ -770,7 +815,31 @@
         <v>medium</v>
       </c>
       <c r="E16" t="str">
-        <v>pending</v>
+        <v>posted</v>
+      </c>
+      <c r="F16" t="str">
+        <v>2026-07-28T16:36:30.544Z</v>
+      </c>
+      <c r="G16" t="str">
+        <v>2026-07-28T16:38:20.227Z</v>
+      </c>
+      <c r="H16" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0015-website-performance-optimization-checklist-improve-speed-wit.md</v>
+      </c>
+      <c r="I16" t="str">
+        <v>approved</v>
+      </c>
+      <c r="J16" t="str">
+        <v>YES 15 / NO 15</v>
+      </c>
+      <c r="K16" t="str">
+        <v>openai/gpt-oss-20b</v>
+      </c>
+      <c r="L16" t="str">
+        <v>28353</v>
+      </c>
+      <c r="M16" t="str">
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28353</v>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
@@ -787,7 +856,22 @@
         <v>long</v>
       </c>
       <c r="E17" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F17" t="str">
+        <v>2026-07-28T16:40:10.574Z</v>
+      </c>
+      <c r="H17" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0016-plan-high-converting-landing-page.md</v>
+      </c>
+      <c r="I17" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J17" t="str">
+        <v>YES 16 / NO 16</v>
+      </c>
+      <c r="K17" t="str">
+        <v>openai/gpt-oss-20b, qwen/qwen2.5-coder-14b</v>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
@@ -804,7 +888,22 @@
         <v>short</v>
       </c>
       <c r="E18" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F18" t="str">
+        <v>2026-07-28T16:41:45.249Z</v>
+      </c>
+      <c r="H18" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0017-landing-page-vs-website-business-needs-each.md</v>
+      </c>
+      <c r="I18" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J18" t="str">
+        <v>YES 17 / NO 17</v>
+      </c>
+      <c r="K18" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
@@ -823,6 +922,9 @@
       <c r="E19" t="str">
         <v>pending</v>
       </c>
+      <c r="I19" t="str">
+        <v>pending</v>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" t="str">
@@ -838,7 +940,22 @@
         <v>long</v>
       </c>
       <c r="E20" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F20" t="str">
+        <v>2026-07-28T15:54:29.639Z</v>
+      </c>
+      <c r="H20" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0019-ecommerce-website-checklist-before-launch.md</v>
+      </c>
+      <c r="I20" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J20" t="str">
+        <v>YES 19 / NO 19</v>
+      </c>
+      <c r="K20" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -855,6 +972,9 @@
         <v>medium</v>
       </c>
       <c r="E21" t="str">
+        <v>error</v>
+      </c>
+      <c r="I21" t="str">
         <v>pending</v>
       </c>
     </row>
@@ -2373,7 +2493,7 @@
       </c>
       <c r="B2" s="1">
         <f>COUNTIF('Blog tracker'!$E$3:$E$52,"pending")</f>
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="C2" t="str">
         <v>Planned words</v>
@@ -4101,27 +4221,27 @@
         <v>A comprehensive article with ten H1 sections for topics that need context, planning, detailed guidance, and evaluation.</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. introduction: Introduce the reader's problem and the guide's outcome.
-2. problem-context: Describe the underlying problem or opportunity.
-3. foundations: Establish definitions and foundational knowledge.
-4. planning: Show how to prepare, scope, or organize the work.
-5. approach-one: Develop the first major part of the solution or evaluation.
-6. approach-two: Develop the second major part of the solution or evaluation.
-7. approach-three: Develop the third major part of the solution or evaluation.
-8. common-mistakes: Identify avoidable mistakes, risks, or weak approaches.
-9. measurement-checklist: Show how to evaluate quality, completion, or results.
+        <v xml:space="preserve">1. introduction: Introduce the reader's problem and the guide's outcome._x000d__x000d_
+2. problem-context: Describe the underlying problem or opportunity._x000d__x000d_
+3. foundations: Establish definitions and foundational knowledge._x000d__x000d_
+4. planning: Show how to prepare, scope, or organize the work._x000d__x000d_
+5. approach-one: Develop the first major part of the solution or evaluation._x000d__x000d_
+6. approach-two: Develop the second major part of the solution or evaluation._x000d__x000d_
+7. approach-three: Develop the third major part of the solution or evaluation._x000d__x000d_
+8. common-mistakes: Identify avoidable mistakes, risks, or weak approaches._x000d__x000d_
+9. measurement-checklist: Show how to evaluate quality, completion, or results._x000d__x000d_
 10. conclusion: Summarize the guide and recommend the most useful next step.</v>
       </c>
       <c r="F2" t="str" xml:space="preserve">
-        <v xml:space="preserve">introduction: 1-3 paragraphs, 35-220 words each
-problem-context: 1-4 paragraphs, 35-220 words each
-foundations: 1-4 paragraphs, 35-220 words each
-planning: 1-4 paragraphs, 35-220 words each
-approach-one: 1-4 paragraphs, 35-220 words each
-approach-two: 1-4 paragraphs, 35-220 words each
-approach-three: 1-4 paragraphs, 35-220 words each
-common-mistakes: 1-4 paragraphs, 35-220 words each
-measurement-checklist: 1-4 paragraphs, 35-220 words each
+        <v xml:space="preserve">introduction: 1-3 paragraphs, 35-220 words each_x000d__x000d_
+problem-context: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+foundations: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+planning: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+approach-one: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+approach-two: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+approach-three: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+common-mistakes: 1-4 paragraphs, 35-220 words each_x000d__x000d_
+measurement-checklist: 1-4 paragraphs, 35-220 words each_x000d__x000d_
 conclusion: 1-3 paragraphs, 35-220 words each</v>
       </c>
       <c r="G2" t="str">
@@ -4148,19 +4268,19 @@
         <v>A balanced article with six H1 sections, enough depth for explanation and implementation guidance.</v>
       </c>
       <c r="E3" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. introduction: Introduce the reader's situation and the article's practical outcome.
-2. foundations: Define the topic and establish the essential background.
-3. key-considerations: Explain the major factors the reader should evaluate.
-4. recommended-approach: Present a practical method, framework, or sequence.
-5. mistakes-and-measurement: Help the reader avoid predictable mistakes and recognize success.
+        <v xml:space="preserve">1. introduction: Introduce the reader's situation and the article's practical outcome._x000d__x000d_
+2. foundations: Define the topic and establish the essential background._x000d__x000d_
+3. key-considerations: Explain the major factors the reader should evaluate._x000d__x000d_
+4. recommended-approach: Present a practical method, framework, or sequence._x000d__x000d_
+5. mistakes-and-measurement: Help the reader avoid predictable mistakes and recognize success._x000d__x000d_
 6. conclusion: Bring the guidance together and recommend a relevant next step.</v>
       </c>
       <c r="F3" t="str" xml:space="preserve">
-        <v xml:space="preserve">introduction: 1-3 paragraphs, 40-240 words each
-foundations: 1-4 paragraphs, 40-240 words each
-key-considerations: 1-4 paragraphs, 40-240 words each
-recommended-approach: 1-4 paragraphs, 40-240 words each
-mistakes-and-measurement: 1-4 paragraphs, 40-240 words each
+        <v xml:space="preserve">introduction: 1-3 paragraphs, 40-240 words each_x000d__x000d_
+foundations: 1-4 paragraphs, 40-240 words each_x000d__x000d_
+key-considerations: 1-4 paragraphs, 40-240 words each_x000d__x000d_
+recommended-approach: 1-4 paragraphs, 40-240 words each_x000d__x000d_
+mistakes-and-measurement: 1-4 paragraphs, 40-240 words each_x000d__x000d_
 conclusion: 1-3 paragraphs, 40-240 words each</v>
       </c>
       <c r="G3" t="str">
@@ -4187,15 +4307,15 @@
         <v>A focused article with four substantial H1 sections and a direct conclusion.</v>
       </c>
       <c r="E4" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. introduction: Introduce the topic, reader problem, and practical promise of the article.
-2. core-explanation: Explain the central idea and why it matters.
-3. practical-guidance: Turn the explanation into practical actions or recommendations.
+        <v xml:space="preserve">1. introduction: Introduce the topic, reader problem, and practical promise of the article._x000d__x000d_
+2. core-explanation: Explain the central idea and why it matters._x000d__x000d_
+3. practical-guidance: Turn the explanation into practical actions or recommendations._x000d__x000d_
 4. conclusion: Summarize the takeaway and give the reader a sensible next step.</v>
       </c>
       <c r="F4" t="str" xml:space="preserve">
-        <v xml:space="preserve">introduction: 1-3 paragraphs, 45-250 words each
-core-explanation: 1-4 paragraphs, 45-250 words each
-practical-guidance: 1-4 paragraphs, 45-250 words each
+        <v xml:space="preserve">introduction: 1-3 paragraphs, 45-250 words each_x000d__x000d_
+core-explanation: 1-4 paragraphs, 45-250 words each_x000d__x000d_
+practical-guidance: 1-4 paragraphs, 45-250 words each_x000d__x000d_
 conclusion: 1-2 paragraphs, 45-250 words each</v>
       </c>
       <c r="G4" t="str">
@@ -4210,6 +4330,7 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I4"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
Record final tracker workflow state
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -920,7 +920,7 @@
         <v>long</v>
       </c>
       <c r="E19" t="str">
-        <v>generating</v>
+        <v>error</v>
       </c>
       <c r="I19" t="str">
         <v>pending</v>
@@ -992,7 +992,22 @@
         <v>long</v>
       </c>
       <c r="E22" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="F22" t="str">
+        <v>2026-07-28T16:47:37.646Z</v>
+      </c>
+      <c r="H22" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0021-website-migration-checklist-relaunch-without-losing-seo.md</v>
+      </c>
+      <c r="I22" t="str">
+        <v>pending</v>
+      </c>
+      <c r="J22" t="str">
+        <v>YES 21 / NO 21</v>
+      </c>
+      <c r="K22" t="str">
+        <v>openai/gpt-oss-20b, qwen/qwen2.5-coder-14b</v>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">

</xml_diff>

<commit_message>
Make blog formats JSON-driven
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -1853,22 +1853,31 @@
         <v>medium</v>
       </c>
       <c r="D53" t="str">
-        <v>awaiting_review</v>
+        <v>posted</v>
       </c>
       <c r="E53" t="str">
         <v>2026-07-29T16:03:59.550Z</v>
       </c>
+      <c r="F53" t="str">
+        <v>2026-07-29T16:07:00.244Z</v>
+      </c>
       <c r="G53" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0052-choose-web-design-company-12-questions.md</v>
       </c>
       <c r="H53" t="str">
-        <v>pending</v>
+        <v>approved</v>
       </c>
       <c r="I53" t="str">
         <v>YES 52 / NO 52</v>
       </c>
       <c r="J53" t="str">
         <v>openai/gpt-oss-20b</v>
+      </c>
+      <c r="K53" t="str">
+        <v>28356</v>
+      </c>
+      <c r="L53" t="str">
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28356</v>
       </c>
     </row>
     <row r="54">
@@ -1882,7 +1891,22 @@
         <v>long</v>
       </c>
       <c r="D54" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E54" t="str">
+        <v>2026-07-29T16:08:17.513Z</v>
+      </c>
+      <c r="G54" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0053-responsive-web-design-best-practices-mobile-first-business-w.md</v>
+      </c>
+      <c r="H54" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I54" t="str">
+        <v>YES 53 / NO 53</v>
+      </c>
+      <c r="J54" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="55">
@@ -1896,7 +1920,22 @@
         <v>long</v>
       </c>
       <c r="D55" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E55" t="str">
+        <v>2026-07-29T16:15:01.606Z</v>
+      </c>
+      <c r="G55" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0054-wordpress-vs-webflow-best-cms-growing-business.md</v>
+      </c>
+      <c r="H55" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I55" t="str">
+        <v>YES 54 / NO 54</v>
+      </c>
+      <c r="J55" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="56">
@@ -3610,7 +3649,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C2:C1000">
-      <formula1>"short,medium,long"</formula1>
+      <formula1>"how-to,long,medium,practical-guidance,short"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Finish blog review and posting fixes
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -1949,7 +1949,31 @@
         <v>long</v>
       </c>
       <c r="D56" t="str">
-        <v>pending</v>
+        <v>posted</v>
+      </c>
+      <c r="E56" t="str">
+        <v>2026-07-29T18:34:54.584Z</v>
+      </c>
+      <c r="F56" t="str">
+        <v>2026-07-29T18:52:44.195Z</v>
+      </c>
+      <c r="G56" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0055-wordpress-vs-squarespace-which-platform-fits-your-business.md</v>
+      </c>
+      <c r="H56" t="str">
+        <v>approved</v>
+      </c>
+      <c r="I56" t="str">
+        <v>YES 55 / NO 55</v>
+      </c>
+      <c r="J56" t="str">
+        <v>openai/gpt-oss-20b</v>
+      </c>
+      <c r="K56" t="str">
+        <v>28357</v>
+      </c>
+      <c r="L56" t="str">
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28357</v>
       </c>
     </row>
     <row r="57">
@@ -1963,7 +1987,22 @@
         <v>long</v>
       </c>
       <c r="D57" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E57" t="str">
+        <v>2026-07-29T18:54:00.132Z</v>
+      </c>
+      <c r="G57" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0056-headless-wordpress-explained-benefits-costs-when-it-makes-se.md</v>
+      </c>
+      <c r="H57" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I57" t="str">
+        <v>YES 56 / NO 56</v>
+      </c>
+      <c r="J57" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="58">
@@ -1977,7 +2016,22 @@
         <v>medium</v>
       </c>
       <c r="D58" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E58" t="str">
+        <v>2026-07-29T19:05:36.781Z</v>
+      </c>
+      <c r="G58" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0057-website-redesign-roi-business-case.md</v>
+      </c>
+      <c r="H58" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I58" t="str">
+        <v>YES 57 / NO 57</v>
+      </c>
+      <c r="J58" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="59">
@@ -1991,7 +2045,22 @@
         <v>medium</v>
       </c>
       <c r="D59" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E59" t="str">
+        <v>2026-07-29T19:07:32.852Z</v>
+      </c>
+      <c r="G59" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0058-website-discovery-phase-guide.md</v>
+      </c>
+      <c r="H59" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I59" t="str">
+        <v>YES 58 / NO 58</v>
+      </c>
+      <c r="J59" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="60">
@@ -2005,7 +2074,22 @@
         <v>long</v>
       </c>
       <c r="D60" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E60" t="str">
+        <v>2026-07-29T20:24:37.237Z</v>
+      </c>
+      <c r="G60" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0059-ux-audit-checklist-find-friction-cost-leads.md</v>
+      </c>
+      <c r="H60" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I60" t="str">
+        <v>YES 59 / NO 59</v>
+      </c>
+      <c r="J60" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="61">

</xml_diff>

<commit_message>
Add holistic article quality review and repair loop
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -2103,7 +2103,22 @@
         <v>short</v>
       </c>
       <c r="D61" t="str">
-        <v>pending</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E61" t="str">
+        <v>2026-07-29T21:09:00.049Z</v>
+      </c>
+      <c r="G61" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0060-mobile-first-web-design-why-businesses-need-it.md</v>
+      </c>
+      <c r="H61" t="str">
+        <v>pending</v>
+      </c>
+      <c r="I61" t="str">
+        <v>YES 60 / NO 60</v>
+      </c>
+      <c r="J61" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="62">

</xml_diff>

<commit_message>
Improve blog quality review and WordPress output
</commit_message>
<xml_diff>
--- a/manual-files/wordpress-blog-content-tracker.xlsx
+++ b/manual-files/wordpress-blog-content-tracker.xlsx
@@ -34,7 +34,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="2">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="200" formatCode="yyyy-mm-dd hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -67,7 +67,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -265,6 +265,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -331,20 +333,23 @@
       <c r="B2" t="str">
         <v>How to build a complete WordPress website from the ground up. This guide explains how WordPress works, how themes and plugins connect, and how key files and folders organize your site’s design, content, features, and functionality.</v>
       </c>
+      <c r="C2" t="str">
+        <v>short</v>
+      </c>
       <c r="D2" t="str">
-        <v>posted</v>
-      </c>
-      <c r="E2" s="1">
-        <v>46230.66897849537</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-07-30T23:33:20.467Z</v>
       </c>
       <c r="F2" s="1">
         <v>46230.6901827662</v>
       </c>
       <c r="G2" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/1-how-to-build-a-complete-wordpress-website-from-the-ground-up-this-guide-explains.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0001-build-wordpress-site-from-scratch.md</v>
       </c>
       <c r="H2" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I2" t="str">
         <v>YES 1 / NO 1</v>
@@ -367,22 +372,22 @@
         <v>Website Redesign Checklist: 15 Steps Before You Hire a Web Design Agency</v>
       </c>
       <c r="C3" t="str">
-        <v>long</v>
+        <v>medium</v>
       </c>
       <c r="D3" t="str">
-        <v>posted</v>
-      </c>
-      <c r="E3" s="1">
-        <v>46231.01608105324</v>
-      </c>
-      <c r="F3" s="1">
-        <v>46231.0247962963</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-07-30T23:36:05.031Z</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-07-30T19:24:40.444Z</v>
       </c>
       <c r="G3" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0002-website-redesign-checklist-15-steps-before-you-hire.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0002-website-redesign-checklist-15-steps-before-hire-agency.md</v>
       </c>
       <c r="H3" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I3" t="str">
         <v>YES 2 / NO 2</v>
@@ -391,10 +396,10 @@
         <v>openai/gpt-oss-20b</v>
       </c>
       <c r="K3" t="str">
-        <v>28351</v>
+        <v>28359</v>
       </c>
       <c r="L3" t="str">
-        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28351</v>
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28359</v>
       </c>
     </row>
     <row r="4">
@@ -405,16 +410,16 @@
         <v>Web Design vs. Web Development: What Growing Businesses Need to Know</v>
       </c>
       <c r="C4" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D4" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E4" s="1">
-        <v>46231.01859716435</v>
+      <c r="E4" t="str">
+        <v>2026-07-30T23:38:45.629Z</v>
       </c>
       <c r="G4" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0003-web-design-vs-web-development.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0003-web-design-vs-web-development-what-growing-businesses-need-t.md</v>
       </c>
       <c r="H4" t="str">
         <v>pending</v>
@@ -434,22 +439,22 @@
         <v>How Much Does a Custom Website Cost? A Practical Budgeting Guide</v>
       </c>
       <c r="C5" t="str">
-        <v>long</v>
+        <v>how-to</v>
       </c>
       <c r="D5" t="str">
-        <v>posted</v>
-      </c>
-      <c r="E5" s="1">
-        <v>46231.080855659726</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-07-30T23:42:29.376Z</v>
       </c>
       <c r="F5" s="1">
         <v>46231.10688986111</v>
       </c>
       <c r="G5" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0004-custom-website-cost-practical-budgeting-guide.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0004-custom-website-cost-practical-budgeting-guide.md</v>
       </c>
       <c r="H5" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I5" t="str">
         <v>YES 4 / NO 4</v>
@@ -472,16 +477,16 @@
         <v>Website Planning Checklist: What to Prepare Before a New Website Project</v>
       </c>
       <c r="C6" t="str">
-        <v>medium</v>
+        <v>practical-guidance</v>
       </c>
       <c r="D6" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E6" s="1">
-        <v>46231.10798234954</v>
+      <c r="E6" t="str">
+        <v>2026-07-30T23:45:07.015Z</v>
       </c>
       <c r="G6" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0005-website-planning-checklist.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0005-website-planning-checklist-what-to-prepare-before-a-new-webs.md</v>
       </c>
       <c r="H6" t="str">
         <v>pending</v>
@@ -506,11 +511,11 @@
       <c r="D7" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E7" s="1">
-        <v>46231.11097840278</v>
+      <c r="E7" t="str">
+        <v>2026-07-30T23:50:16.938Z</v>
       </c>
       <c r="G7" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0006-conversion-focused-website-design.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0006-conversion-focused-website-design-turn-visitors-into-leads.md</v>
       </c>
       <c r="H7" t="str">
         <v>pending</v>
@@ -530,16 +535,16 @@
         <v>B2B Website Design Best Practices for Clearer Buying Journeys</v>
       </c>
       <c r="C8" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D8" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E8" s="1">
-        <v>46231.11300480324</v>
+      <c r="E8" t="str">
+        <v>2026-07-30T23:52:28.099Z</v>
       </c>
       <c r="G8" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0007-b2b-website-design-best-practices.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0007-b2b-website-design-best-practices-clearer-buying-journeys.md</v>
       </c>
       <c r="H8" t="str">
         <v>pending</v>
@@ -559,16 +564,16 @@
         <v>Website Navigation Best Practices: Build Menus That Help Users Convert</v>
       </c>
       <c r="C9" t="str">
-        <v>short</v>
+        <v>long</v>
       </c>
       <c r="D9" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E9" s="1">
-        <v>46231.1144415625</v>
+      <c r="E9" t="str">
+        <v>2026-07-30T23:54:58.819Z</v>
       </c>
       <c r="G9" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0008-website-navigation-best-practices-build-menus-that-help-user.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0008-website-navigation-best-practices-build-menus-that-help-user.md</v>
       </c>
       <c r="H9" t="str">
         <v>pending</v>
@@ -588,16 +593,16 @@
         <v>Website Accessibility Checklist for Business Websites</v>
       </c>
       <c r="C10" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D10" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E10" s="1">
-        <v>46231.116490914355</v>
+      <c r="E10" t="str">
+        <v>2026-07-30T23:58:30.060Z</v>
       </c>
       <c r="G10" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0009-website-accessibility-checklist-business-websites.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0009-website-accessibility-checklist-business-websites.md</v>
       </c>
       <c r="H10" t="str">
         <v>pending</v>
@@ -622,11 +627,11 @@
       <c r="D11" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E11" s="1">
-        <v>46231.11876748843</v>
+      <c r="E11" t="str">
+        <v>2026-07-31T00:01:19.214Z</v>
       </c>
       <c r="G11" t="str">
-        <v>/Users/grasshopper/Developer/repos/WP-blog-agent/data/drafts/blog-0010-custom-wordpress-development-vs-page-builders.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0010-custom-wordpress-development-vs-page-builders.md</v>
       </c>
       <c r="H11" t="str">
         <v>pending</v>
@@ -649,10 +654,22 @@
         <v>long</v>
       </c>
       <c r="D12" t="str">
-        <v>generating</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E12" t="str">
+        <v>2026-07-31T00:04:23.873Z</v>
+      </c>
+      <c r="G12" t="str">
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0011-wordpress-maintenance-checklist-updates-backups-security-per.md</v>
       </c>
       <c r="H12" t="str">
         <v>pending</v>
+      </c>
+      <c r="I12" t="str">
+        <v>YES 11 / NO 11</v>
+      </c>
+      <c r="J12" t="str">
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="13">
@@ -663,16 +680,16 @@
         <v>How to Choose a WordPress Development Agency for a Business Website</v>
       </c>
       <c r="C13" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D13" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E13" s="1">
-        <v>46231.651349293985</v>
+      <c r="E13" t="str">
+        <v>2026-07-31T00:07:19.039Z</v>
       </c>
       <c r="G13" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0012-choose-wordpress-development-agency.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0012-choose-wordpress-development-agency-for-business-website.md</v>
       </c>
       <c r="H13" t="str">
         <v>pending</v>
@@ -692,13 +709,13 @@
         <v>WordPress Security Best Practices for Business Websites</v>
       </c>
       <c r="C14" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D14" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E14" s="1">
-        <v>46231.65331533565</v>
+      <c r="E14" t="str">
+        <v>2026-07-31T00:09:59.958Z</v>
       </c>
       <c r="G14" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0013-wordpress-security-best-practices-business-websites.md</v>
@@ -726,11 +743,11 @@
       <c r="D15" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E15" s="1">
-        <v>46231.65519037037</v>
+      <c r="E15" t="str">
+        <v>2026-07-31T00:13:23.581Z</v>
       </c>
       <c r="G15" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0014-wordpress-website-faster-core-web-vitals-guide.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0014-make-wordpress-website-faster-core-web-vitals-guide.md</v>
       </c>
       <c r="H15" t="str">
         <v>pending</v>
@@ -750,22 +767,22 @@
         <v>Website Performance Optimization Checklist: Improve Speed Without Breaking Your Site</v>
       </c>
       <c r="C16" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D16" t="str">
-        <v>posted</v>
-      </c>
-      <c r="E16" s="1">
-        <v>46231.69202018518</v>
+        <v>awaiting_review</v>
+      </c>
+      <c r="E16" t="str">
+        <v>2026-07-31T00:17:07.345Z</v>
       </c>
       <c r="F16" s="1">
         <v>46231.69328966435</v>
       </c>
       <c r="G16" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0015-website-performance-optimization-checklist-improve-speed-wit.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0015-website-performance-optimization-checklist.md</v>
       </c>
       <c r="H16" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I16" t="str">
         <v>YES 15 / NO 15</v>
@@ -793,11 +810,11 @@
       <c r="D17" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E17" s="1">
-        <v>46231.6945668287</v>
+      <c r="E17" t="str">
+        <v>2026-07-31T00:22:18.426Z</v>
       </c>
       <c r="G17" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0016-plan-high-converting-landing-page.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0016-how-to-plan-a-high-converting-landing-page.md</v>
       </c>
       <c r="H17" t="str">
         <v>pending</v>
@@ -806,7 +823,7 @@
         <v>YES 16 / NO 16</v>
       </c>
       <c r="J17" t="str">
-        <v>openai/gpt-oss-20b, qwen/qwen2.5-coder-14b</v>
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="18">
@@ -817,16 +834,16 @@
         <v>Landing Page vs. Website: When Your Business Needs Each</v>
       </c>
       <c r="C18" t="str">
-        <v>short</v>
+        <v>long</v>
       </c>
       <c r="D18" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E18" s="1">
-        <v>46231.695662604165</v>
+      <c r="E18" t="str">
+        <v>2026-07-31T00:25:32.288Z</v>
       </c>
       <c r="G18" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0017-landing-page-vs-website-business-needs-each.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0017-landing-page-vs-website-when-your-business-needs-each.md</v>
       </c>
       <c r="H18" t="str">
         <v>pending</v>
@@ -852,10 +869,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E19" t="str">
-        <v>2026-07-29T12:09:16.549Z</v>
+        <v>2026-07-31T00:29:39.739Z</v>
       </c>
       <c r="G19" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0018-woocommerce-vs-shopify-choosing-right-ecommerce-platform.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0018-woocommerce-vs-shopify-choosing-the-right-ecommerce-platform.md</v>
       </c>
       <c r="H19" t="str">
         <v>pending</v>
@@ -880,11 +897,11 @@
       <c r="D20" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E20" s="1">
-        <v>46231.66284304398</v>
+      <c r="E20" t="str">
+        <v>2026-07-31T00:34:18.845Z</v>
       </c>
       <c r="G20" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0019-ecommerce-website-checklist-before-launch.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0019-ecommerce-website-checklist-plan-before-launch.md</v>
       </c>
       <c r="H20" t="str">
         <v>pending</v>
@@ -904,16 +921,16 @@
         <v>Ecommerce Product Page Best Practices That Support More Sales</v>
       </c>
       <c r="C21" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D21" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E21" t="str">
-        <v>2026-07-29T13:36:05.740Z</v>
+        <v>2026-07-31T00:37:52.433Z</v>
       </c>
       <c r="G21" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0020-ecommerce-product-page-best-practices.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0020-ecommerce-product-page-best-practices-that-support-more-sale.md</v>
       </c>
       <c r="H21" t="str">
         <v>pending</v>
@@ -938,11 +955,11 @@
       <c r="D22" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E22" s="1">
-        <v>46231.69974127315</v>
+      <c r="E22" t="str">
+        <v>2026-07-31T00:41:19.859Z</v>
       </c>
       <c r="G22" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0021-website-migration-checklist-relaunch-without-losing-seo.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0021-website-migration-checklist-how-to-relaunch-without-losing-s.md</v>
       </c>
       <c r="H22" t="str">
         <v>pending</v>
@@ -951,7 +968,7 @@
         <v>YES 21 / NO 21</v>
       </c>
       <c r="J22" t="str">
-        <v>openai/gpt-oss-20b, qwen/qwen2.5-coder-14b</v>
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="23">
@@ -962,13 +979,13 @@
         <v>How to Measure Website Conversion Rate and Find Drop-Off Points</v>
       </c>
       <c r="C23" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D23" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E23" t="str">
-        <v>2026-07-29T13:37:55.192Z</v>
+        <v>2026-07-31T00:44:07.753Z</v>
       </c>
       <c r="G23" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0022-measure-website-conversion-rate-drop-off-points.md</v>
@@ -991,16 +1008,16 @@
         <v>Website Analytics for Small Businesses: Metrics That Actually Matter</v>
       </c>
       <c r="C24" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D24" t="str">
         <v>awaiting_review</v>
       </c>
-      <c r="E24" s="1">
-        <v>46231.73590177084</v>
+      <c r="E24" t="str">
+        <v>2026-07-31T00:47:49.392Z</v>
       </c>
       <c r="G24" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0023-website-analytics-small-business-metrics-that-matter.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0023-website-analytics-small-business-metrics-that-actually-matte.md</v>
       </c>
       <c r="H24" t="str">
         <v>pending</v>
@@ -1009,7 +1026,7 @@
         <v>YES 23 / NO 23</v>
       </c>
       <c r="J24" t="str">
-        <v>openai/gpt-oss-20b, qwen/qwen2.5-coder-14b</v>
+        <v>openai/gpt-oss-20b</v>
       </c>
     </row>
     <row r="25">
@@ -1026,10 +1043,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E25" t="str">
-        <v>2026-07-29T13:40:12.859Z</v>
+        <v>2026-07-31T00:51:36.476Z</v>
       </c>
       <c r="G25" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0024-website-content-strategy-sales.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0024-website-content-strategy-supports-sales.md</v>
       </c>
       <c r="H25" t="str">
         <v>pending</v>
@@ -1049,13 +1066,13 @@
         <v>Web Design Brief Template: What to Include Before Your Project Starts</v>
       </c>
       <c r="C26" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D26" t="str">
-        <v>awaiting_review</v>
+        <v>error</v>
       </c>
       <c r="E26" t="str">
-        <v>2026-07-29T13:42:01.156Z</v>
+        <v>2026-07-31T00:54:55.112Z</v>
       </c>
       <c r="G26" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0025-web-design-brief-template-before-project-starts.md</v>
@@ -1084,10 +1101,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E27" t="str">
-        <v>2026-07-29T13:44:17.970Z</v>
+        <v>2026-07-31T00:58:40.894Z</v>
       </c>
       <c r="G27" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0026-workflow-automation-ideas-10-manual-processes.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0026-workflow-automation-ideas-10-manual-processes-businesses-can.md</v>
       </c>
       <c r="H27" t="str">
         <v>pending</v>
@@ -1107,16 +1124,16 @@
         <v>What Is Workflow Automation? A Practical Guide for Growing Teams</v>
       </c>
       <c r="C28" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D28" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E28" t="str">
-        <v>2026-07-29T13:46:07.481Z</v>
+        <v>2026-07-31T01:01:50.778Z</v>
       </c>
       <c r="G28" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0027-workflow-automation-practical-guide-growing-teams.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0027-what-is-workflow-automation-practical-guide-for-growing-team.md</v>
       </c>
       <c r="H28" t="str">
         <v>pending</v>
@@ -1139,7 +1156,7 @@
         <v>long</v>
       </c>
       <c r="D29" t="str">
-        <v>awaiting_review</v>
+        <v>error</v>
       </c>
       <c r="E29" t="str">
         <v>2026-07-29T13:48:20.187Z</v>
@@ -1171,7 +1188,7 @@
         <v>awaiting_review</v>
       </c>
       <c r="E30" t="str">
-        <v>2026-07-29T13:50:34.743Z</v>
+        <v>2026-07-31T01:15:33.220Z</v>
       </c>
       <c r="G30" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0029-custom-crm-development-when-tailored-system-makes-sense.md</v>
@@ -1194,13 +1211,13 @@
         <v>API Integration for Businesses: What It Is and When You Need It</v>
       </c>
       <c r="C31" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D31" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E31" t="str">
-        <v>2026-07-29T13:52:21.221Z</v>
+        <v>2026-07-31T01:36:09.416Z</v>
       </c>
       <c r="G31" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0030-api-integration-for-businesses-what-it-is-and-when-you-need-.md</v>
@@ -1223,13 +1240,13 @@
         <v>Internal Tools for Businesses: How Custom Admin Dashboards Save Time</v>
       </c>
       <c r="C32" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D32" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E32" t="str">
-        <v>2026-07-29T13:54:07.623Z</v>
+        <v>2026-07-31T01:39:24.591Z</v>
       </c>
       <c r="G32" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0031-internal-tools-custom-admin-dashboards-save-time.md</v>
@@ -1258,10 +1275,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E33" t="str">
-        <v>2026-07-29T13:56:17.786Z</v>
+        <v>2026-07-31T01:42:16.916Z</v>
       </c>
       <c r="G33" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0032-bpa-best-first-project.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0032-business-process-automation-best-first-project.md</v>
       </c>
       <c r="H33" t="str">
         <v>pending</v>
@@ -1287,7 +1304,7 @@
         <v>awaiting_review</v>
       </c>
       <c r="E34" t="str">
-        <v>2026-07-29T13:58:35.142Z</v>
+        <v>2026-07-31T01:45:41.559Z</v>
       </c>
       <c r="G34" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0033-custom-software-development-process-discovery-launch.md</v>
@@ -1313,22 +1330,31 @@
         <v>long</v>
       </c>
       <c r="D35" t="str">
-        <v>awaiting_review</v>
+        <v>posted</v>
       </c>
       <c r="E35" t="str">
-        <v>2026-07-29T14:00:48.473Z</v>
+        <v>2026-07-31T01:49:20.358Z</v>
+      </c>
+      <c r="F35" t="str">
+        <v>2026-07-31T02:01:43.768Z</v>
       </c>
       <c r="G35" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0034-mobile-app-development-process-idea-to-launch.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0034-mobile-app-development-process-from-idea-to-app-store-launch.md</v>
       </c>
       <c r="H35" t="str">
-        <v>pending</v>
+        <v>approved</v>
       </c>
       <c r="I35" t="str">
         <v>YES 34 / NO 34</v>
       </c>
       <c r="J35" t="str">
         <v>openai/gpt-oss-20b</v>
+      </c>
+      <c r="K35" t="str">
+        <v>28360</v>
+      </c>
+      <c r="L35" t="str">
+        <v>https://6-22-shop-grasshoppergardens-press-cache.mystagingwebsite.com/?p=28360</v>
       </c>
     </row>
     <row r="36">
@@ -1345,7 +1371,7 @@
         <v>awaiting_review</v>
       </c>
       <c r="E36" t="str">
-        <v>2026-07-29T14:03:01.369Z</v>
+        <v>2026-07-31T01:52:18.108Z</v>
       </c>
       <c r="G36" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0035-native-vs-cross-platform-app-development-which-should-you-ch.md</v>
@@ -1368,10 +1394,10 @@
         <v>How to Scope an MVP App Without Losing the Core Idea</v>
       </c>
       <c r="C37" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D37" t="str">
-        <v>awaiting_review</v>
+        <v>error</v>
       </c>
       <c r="E37" t="str">
         <v>2026-07-29T14:04:50.474Z</v>
@@ -1397,16 +1423,16 @@
         <v>Mobile Payment Integration: What Businesses Need to Plan For</v>
       </c>
       <c r="C38" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D38" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E38" t="str">
-        <v>2026-07-29T14:06:37.717Z</v>
+        <v>2026-07-31T02:00:25.997Z</v>
       </c>
       <c r="G38" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0037-mobile-payment-integration-what-businesses-need-to-plan-for.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0037-mobile-payment-integration-planning.md</v>
       </c>
       <c r="H38" t="str">
         <v>pending</v>
@@ -1426,13 +1452,13 @@
         <v>Push Notification Best Practices: How to Increase App Engagement</v>
       </c>
       <c r="C39" t="str">
-        <v>short</v>
+        <v>long</v>
       </c>
       <c r="D39" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E39" t="str">
-        <v>2026-07-29T14:08:15.500Z</v>
+        <v>2026-07-31T02:04:57.812Z</v>
       </c>
       <c r="G39" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0038-push-notification-best-practices-increase-app-engagement.md</v>
@@ -1455,13 +1481,13 @@
         <v>Mobile App Analytics: Key Metrics to Track After Launch</v>
       </c>
       <c r="C40" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D40" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E40" t="str">
-        <v>2026-07-29T14:10:01.638Z</v>
+        <v>2026-07-31T02:08:56.900Z</v>
       </c>
       <c r="G40" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0039-mobile-app-analytics-key-metrics-after-launch.md</v>
@@ -1484,16 +1510,16 @@
         <v>App Maintenance Checklist: What Happens After Your App Launches</v>
       </c>
       <c r="C41" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D41" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E41" t="str">
-        <v>2026-07-29T14:11:46.559Z</v>
+        <v>2026-07-31T02:12:33.805Z</v>
       </c>
       <c r="G41" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0040-app-maintenance-checklist-after-launch.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0040-app-maintenance-checklist-what-happens-after-your-app-launch.md</v>
       </c>
       <c r="H41" t="str">
         <v>pending</v>
@@ -1519,10 +1545,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E42" t="str">
-        <v>2026-07-29T14:13:53.886Z</v>
+        <v>2026-07-31T02:15:27.591Z</v>
       </c>
       <c r="G42" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0041-technical-seo-audit-checklist-first-review.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0041-technical-seo-audit-checklist-review-first.md</v>
       </c>
       <c r="H42" t="str">
         <v>pending</v>
@@ -1542,16 +1568,16 @@
         <v>What Is Schema Markup and How Does It Help Your Website?</v>
       </c>
       <c r="C43" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D43" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E43" t="str">
-        <v>2026-07-29T14:15:41.404Z</v>
+        <v>2026-07-31T02:18:29.098Z</v>
       </c>
       <c r="G43" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0042-schema-markup-website-benefits.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0042-what-is-schema-markup-and-how-does-it-help-your-website.md</v>
       </c>
       <c r="H43" t="str">
         <v>pending</v>
@@ -1571,13 +1597,13 @@
         <v>How to Improve Website Indexing: A Practical Google Search Console Guide</v>
       </c>
       <c r="C44" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D44" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E44" t="str">
-        <v>2026-07-29T14:17:26.602Z</v>
+        <v>2026-07-31T02:21:24.813Z</v>
       </c>
       <c r="G44" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0043-improve-website-indexing-google-search-console-guide.md</v>
@@ -1600,16 +1626,16 @@
         <v>Crawl Budget Explained: When It Matters and How to Improve Crawlability</v>
       </c>
       <c r="C45" t="str">
-        <v>short</v>
+        <v>long</v>
       </c>
       <c r="D45" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E45" t="str">
-        <v>2026-07-29T14:19:01.458Z</v>
+        <v>2026-07-31T02:24:57.419Z</v>
       </c>
       <c r="G45" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0044-crawl-budget-explained-improve-crawlability.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0044-crawl-budget-explained-when-it-matters-how-to-improve-crawla.md</v>
       </c>
       <c r="H45" t="str">
         <v>pending</v>
@@ -1635,10 +1661,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E46" t="str">
-        <v>2026-07-29T14:21:12.494Z</v>
+        <v>2026-07-31T02:29:01.279Z</v>
       </c>
       <c r="G46" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0045-local-seo-checklist-service-businesses.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0045-local-seo-checklist-for-service-businesses.md</v>
       </c>
       <c r="H46" t="str">
         <v>pending</v>
@@ -1664,10 +1690,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E47" t="str">
-        <v>2026-07-29T14:23:30.850Z</v>
+        <v>2026-07-31T02:32:21.834Z</v>
       </c>
       <c r="G47" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0046-seo-website-migration-checklist-protect-rankings.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0046-seo-website-migration-checklist-protect-rankings-during-rede.md</v>
       </c>
       <c r="H47" t="str">
         <v>pending</v>
@@ -1687,16 +1713,16 @@
         <v>Internal Linking Strategy for SEO: How to Connect Service Pages and Blog Content</v>
       </c>
       <c r="C48" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D48" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E48" t="str">
-        <v>2026-07-29T14:25:25.443Z</v>
+        <v>2026-07-31T02:35:25.149Z</v>
       </c>
       <c r="G48" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0047-internal-linking-strategy-service-pages-blog-content.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0047-internal-linking-strategy-seo-connect-service-pages-blog-con.md</v>
       </c>
       <c r="H48" t="str">
         <v>pending</v>
@@ -1716,16 +1742,16 @@
         <v>Core Web Vitals for SEO: What They Mean for Business Websites</v>
       </c>
       <c r="C49" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D49" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E49" t="str">
-        <v>2026-07-29T14:27:12.563Z</v>
+        <v>2026-07-31T02:39:27.829Z</v>
       </c>
       <c r="G49" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0048-core-web-vitals-seo-business-websites.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0048-core-web-vitals-for-seo-what-they-mean-for-business-websites.md</v>
       </c>
       <c r="H49" t="str">
         <v>pending</v>
@@ -1745,13 +1771,13 @@
         <v>GA4 Setup Checklist for a New Website</v>
       </c>
       <c r="C50" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D50" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E50" t="str">
-        <v>2026-07-29T14:28:58.972Z</v>
+        <v>2026-07-31T02:42:53.266Z</v>
       </c>
       <c r="G50" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0049-ga4-setup-checklist-new-website.md</v>
@@ -1774,22 +1800,22 @@
         <v>Google Tag Manager Setup Guide: A Clean Foundation for Reliable Tracking</v>
       </c>
       <c r="C51" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D51" t="str">
-        <v>posted</v>
+        <v>awaiting_review</v>
       </c>
       <c r="E51" t="str">
-        <v>2026-07-29T14:30:46.463Z</v>
+        <v>2026-07-31T02:45:55.318Z</v>
       </c>
       <c r="F51" t="str">
         <v>2026-07-29T15:17:11.689Z</v>
       </c>
       <c r="G51" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0050-google-tag-manager-setup-guide-clean-foundation.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0050-google-tag-manager-setup-guide-clean-foundation-reliable-tra.md</v>
       </c>
       <c r="H51" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I51" t="str">
         <v>YES 50 / NO 50</v>
@@ -1812,22 +1838,22 @@
         <v>How to Audit GA4: Find Tracking Errors Before They Affect Decisions</v>
       </c>
       <c r="C52" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D52" t="str">
-        <v>posted</v>
+        <v>awaiting_review</v>
       </c>
       <c r="E52" t="str">
-        <v>2026-07-29T14:32:34.345Z</v>
+        <v>2026-07-31T02:50:51.779Z</v>
       </c>
       <c r="F52" t="str">
         <v>2026-07-29T15:15:55.928Z</v>
       </c>
       <c r="G52" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0051-audit-ga4-find-tracking-errors.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0051-audit-ga4-find-tracking-errors-before-they-affect-decisions.md</v>
       </c>
       <c r="H52" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I52" t="str">
         <v>YES 51 / NO 51</v>
@@ -1850,13 +1876,13 @@
         <v>How to Choose a Web Design Company: 12 Questions to Ask Before You Hire</v>
       </c>
       <c r="C53" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D53" t="str">
-        <v>posted</v>
+        <v>awaiting_review</v>
       </c>
       <c r="E53" t="str">
-        <v>2026-07-29T16:03:59.550Z</v>
+        <v>2026-07-31T02:54:45.355Z</v>
       </c>
       <c r="F53" t="str">
         <v>2026-07-29T16:07:00.244Z</v>
@@ -1865,7 +1891,7 @@
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0052-choose-web-design-company-12-questions.md</v>
       </c>
       <c r="H53" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I53" t="str">
         <v>YES 52 / NO 52</v>
@@ -1894,7 +1920,7 @@
         <v>awaiting_review</v>
       </c>
       <c r="E54" t="str">
-        <v>2026-07-29T16:08:17.513Z</v>
+        <v>2026-07-31T02:58:52.655Z</v>
       </c>
       <c r="G54" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0053-responsive-web-design-best-practices-mobile-first-business-w.md</v>
@@ -1923,10 +1949,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E55" t="str">
-        <v>2026-07-29T16:15:01.606Z</v>
+        <v>2026-07-31T03:03:18.018Z</v>
       </c>
       <c r="G55" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0054-wordpress-vs-webflow-best-cms-growing-business.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0054-wordpress-vs-webflow-cms-for-growing-business.md</v>
       </c>
       <c r="H55" t="str">
         <v>pending</v>
@@ -1949,10 +1975,10 @@
         <v>long</v>
       </c>
       <c r="D56" t="str">
-        <v>posted</v>
+        <v>awaiting_review</v>
       </c>
       <c r="E56" t="str">
-        <v>2026-07-29T18:34:54.584Z</v>
+        <v>2026-07-31T03:06:52.193Z</v>
       </c>
       <c r="F56" t="str">
         <v>2026-07-29T18:52:44.195Z</v>
@@ -1961,7 +1987,7 @@
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0055-wordpress-vs-squarespace-which-platform-fits-your-business.md</v>
       </c>
       <c r="H56" t="str">
-        <v>approved</v>
+        <v>pending</v>
       </c>
       <c r="I56" t="str">
         <v>YES 55 / NO 55</v>
@@ -1990,7 +2016,7 @@
         <v>awaiting_review</v>
       </c>
       <c r="E57" t="str">
-        <v>2026-07-29T18:54:00.132Z</v>
+        <v>2026-07-31T03:10:59.938Z</v>
       </c>
       <c r="G57" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0056-headless-wordpress-explained-benefits-costs-when-it-makes-se.md</v>
@@ -2013,13 +2039,13 @@
         <v>Website Redesign ROI: How to Build a Business Case for a Better Website</v>
       </c>
       <c r="C58" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D58" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E58" t="str">
-        <v>2026-07-29T19:05:36.781Z</v>
+        <v>2026-07-31T03:15:00.746Z</v>
       </c>
       <c r="G58" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0057-website-redesign-roi-business-case.md</v>
@@ -2042,13 +2068,13 @@
         <v>What Is a Website Discovery Phase? A Guide to Strategy Before Design</v>
       </c>
       <c r="C59" t="str">
-        <v>medium</v>
+        <v>long</v>
       </c>
       <c r="D59" t="str">
         <v>awaiting_review</v>
       </c>
       <c r="E59" t="str">
-        <v>2026-07-29T19:07:32.852Z</v>
+        <v>2026-07-31T03:18:00.130Z</v>
       </c>
       <c r="G59" t="str">
         <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0058-website-discovery-phase-guide.md</v>
@@ -2077,10 +2103,10 @@
         <v>awaiting_review</v>
       </c>
       <c r="E60" t="str">
-        <v>2026-07-29T20:24:37.237Z</v>
+        <v>2026-07-31T03:21:35.311Z</v>
       </c>
       <c r="G60" t="str">
-        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0059-ux-audit-checklist-find-friction-cost-leads.md</v>
+        <v>/Users/dev/Developer/repos/WP-blog-agent/data/drafts/blog-0059-ux-audit-checklist-find-friction-costs-leads.md</v>
       </c>
       <c r="H60" t="str">
         <v>pending</v>
@@ -2100,10 +2126,10 @@
         <v>Mobile-First Web Design: What It Means and Why Businesses Need It</v>
       </c>
       <c r="C61" t="str">
-        <v>short</v>
+        <v>long</v>
       </c>
       <c r="D61" t="str">
-        <v>awaiting_review</v>
+        <v>generating</v>
       </c>
       <c r="E61" t="str">
         <v>2026-07-29T21:09:00.049Z</v>

</xml_diff>